<commit_message>
Fix CVE-2025-54068 preconditions to match the rebuilt (authenticated) lab
The 54068 lab rebuild (6dc8737) moved exploitation to the real authenticated Snipe-IT
PersonalAccessTokens sink at /account/api and removed the synthetic unauth /demo
component, but the metadata preconditions still described the old /demo path. Updated the
Auth + Network preconditions to state: detection runs unauthenticated (not_detected),
exploitation requires seeded staff creds, real sink is auth-gated. Workbook re-synced; 170/170.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lvcscan/docs/Laravel_Vulnerabilities.xlsx
+++ b/lvcscan/docs/Laravel_Vulnerabilities.xlsx
@@ -2203,10 +2203,10 @@
       </c>
       <c r="N13" s="23" t="inlineStr">
         <is>
-          <t>Auth: Unauthenticated by CVE class, and the deployed lab matches it — the vulnerable sink (untyped `public $name` on App\Livewire\PublicDemo) is mounted on the PUBLIC `/demo` route with web middleware only (no auth), so the RCE is reachable with NO credentials. Seeded creds are OPTIONAL (only for the authenticated PersonalAccessTokens fallback path); no APP_KEY required.
+          <t>Auth: AUTHENTICATED against this lab. The lab now exploits the REAL stock Snipe-IT sink — the untyped `public $name` on App\Livewire\PersonalAccessTokens at the authenticated route /account/api (the synthetic unauthenticated /demo component was removed for realism). Detection runs unauthenticated (finds no reachable component -&gt; not_detected); exploitation requires seeded staff creds (-U admin -P Password123!). The Livewire hydration bug is unauthenticated by CVE class, but the genuine Snipe-IT surface is auth-gated. No APP_KEY required.
 Affected version: Reachable Livewire v3 component, versions 3.0.0-beta.1 through 3.6.3 (fixed in 3.6.4)
 Config: Component has at least one untyped/weakly-typed public property (e.g. public $count = 0;); a scalar type hint such as public int $count closes the hole
-Network: Attacker must reach the vulnerable Livewire component/update HTTP(S) endpoint. The lab exposes this unauthenticated at /demo (web middleware only); the scanner probes the public surface first and only uses seeded auth if credentials are supplied. The exploit trigger and proof are in-band HTTP, not OOB.
+Network: Attacker must authenticate to Snipe-IT and reach the real Livewire component at /account/api (the module logs in with -U/-P, fetches the component snapshot, and sends the malicious hydration update). The exploit trigger and proof are in-band HTTP, not OOB.
 Lab rebuild: `bash vuln-labs/apps/snipe-it/8.1.18/cve-2025-54068_auth-deserialize-rce_41004-42004/run.sh`; module `modules/cves/cve_2025_54068.py`; Snipe-IT 8.1.18 with vulnerable Livewire v3 component on php:8.2-apache; seeded admin `admin` / `Password123!` (optional, for the authed fallback path); vulnerable/hardened HTTP ports 41004/42004.
 Flags:
 - Requires Auth (detect): No

</xml_diff>

<commit_message>
Add missing CVE-2016-10074 row to the workbook (completeness)
The sheet had 29 rows while check.py --list ships 30 CVEs; CVE-2016-10074 was absent.
Added an honest row: swiftmailer_dependency_rce, Critical, no dedicated lab, Component
noting it is a SwiftMailer transport CVE bundled by legacy Laravel (not Laravel core),
preconditions synced from metadata. Sheet now 30/30 with zero precondition drift; 170/170.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lvcscan/docs/Laravel_Vulnerabilities.xlsx
+++ b/lvcscan/docs/Laravel_Vulnerabilities.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y30"/>
+  <dimension ref="A1:Y31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="16.38" customWidth="1" style="22" min="1" max="1"/>
@@ -4537,6 +4537,88 @@
         </is>
       </c>
       <c r="Y30" s="23" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t>CVE-2016-10074</t>
+        </is>
+      </c>
+      <c r="E31" s="0" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F31" s="0" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="H31" s="0" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="I31" s="0" t="inlineStr">
+        <is>
+          <t>Dependency upgrade</t>
+        </is>
+      </c>
+      <c r="J31" s="0" t="inlineStr">
+        <is>
+          <t>SwiftMailer (mail transport bundled by legacy Laravel 4.x/5.0) — NOT Laravel core</t>
+        </is>
+      </c>
+      <c r="K31" s="0" t="inlineStr">
+        <is>
+          <t>[SwiftMailer package CVE (&lt;5.4.5), NOT Laravel core. Needs old Laravel with sendmail transport plus attacker-controlled From. No lab present.] SwiftMailer sendmail argument-injection RCE</t>
+        </is>
+      </c>
+      <c r="N31" s="0" t="inlineStr">
+        <is>
+          <t>Auth: Unauthenticated; no APP_KEY required.
+Affected version: SwiftMailer &lt;= 5.4.4 when Laravel or another PHP app uses the vulnerable sendmail/mail transport.
+Config: A reachable mail-sending endpoint passes attacker-controlled From/Sender/Return-Path data into SwiftMailer sendmail transport.
+Network: Attacker must reach the HTTP(S) mail-send proof endpoint. Exploitation injects sendmail arguments through the email reverse-path and reads the written proof file over HTTP; no APP_KEY, callback, or external OOB channel is required.
+Flags:
+- Requires Auth (detect): No
+- Command Capable: Yes
+- APP_KEY Required: No</t>
+        </is>
+      </c>
+      <c r="P31" s="0" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q31" s="0" t="inlineStr">
+        <is>
+          <t>No dedicated lab (SwiftMailer package CVE; not reproducible against stock Laravel)</t>
+        </is>
+      </c>
+      <c r="R31" s="0" t="inlineStr">
+        <is>
+          <t>modules/cves/cve_2016_10074.py</t>
+        </is>
+      </c>
+      <c r="S31" s="0" t="inlineStr">
+        <is>
+          <t>modules/cves/cve_2016_10074.py</t>
+        </is>
+      </c>
+      <c r="T31" s="0" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U31" s="0" t="inlineStr">
+        <is>
+          <t>No dedicated lab; not run</t>
+        </is>
+      </c>
+      <c r="Y31" s="0" t="inlineStr">
+        <is>
+          <t>Added for completeness: ships in check.py --list but was absent from the sheet. SwiftMailer &lt;5.4.5 sendmail arg-injection RCE; requires old Laravel with the sendmail/mail transport + attacker-controlled From. Reclassified swiftmailer_dependency_rce.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="11">

</xml_diff>